<commit_message>
Actualiza nota de verificacion en Analisis_Escenarios_Lote75
</commit_message>
<xml_diff>
--- a/Analisis_Escenarios/Analisis_Escenarios_Lote75.xlsx
+++ b/Analisis_Escenarios/Analisis_Escenarios_Lote75.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Parametros" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Escenario_Lote75" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Riesgo_Trabajo_Desplazado" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Detalle_Grupos_Secuencia" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Verificacion_vs_Madelyn" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parametros" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenario_Lote75" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riesgo_Trabajo_Desplazado" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle_Grupos_Secuencia" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verificacion_vs_Madelyn" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2557,7 +2557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2739,12 +2739,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Estos valores se recalcularon desde 'Simio Aerospace Data.xlsx' de forma</t>
+          <t>Estos valores se recalcularon de forma independiente desde</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>independiente al archivo de Madelyn, como control de calidad.</t>
+          <t>'Simio Aerospace Data.xlsx', como control de calidad, y coinciden en</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -2755,22 +2755,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Coinciden con Analisis_Capacidad.xlsx en todas las celdas salvo WorkCell5</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>(ver nota de calidad en docs/00_contexto_y_plan.md sobre el Calculo 3 de esa hoja).</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+          <t>todas las celdas con los valores de Analisis_Capacidad.xlsx.</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>